<commit_message>
Complete LOOCV regime with Val for BoostStack + GB_seed_ensemble
</commit_message>
<xml_diff>
--- a/Slump_ML_Results_v2.xlsx
+++ b/Slump_ML_Results_v2.xlsx
@@ -80,7 +80,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -102,11 +102,55 @@
         <color rgb="00999999"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -144,6 +188,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -526,8 +578,11 @@
           <t>DATASET OVERVIEW — SLUMP DATA</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -859,7 +914,6 @@
         <v>129.9889</v>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
@@ -960,14 +1014,33 @@
           <t>SVR (RBF) — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -975,16 +1048,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -1897,7 +1976,6 @@
         <v>2.308</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -2048,14 +2126,22 @@
         <v>153.2297</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2063,16 +2149,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -2158,7 +2250,7 @@
         <v>180</v>
       </c>
       <c r="C76" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E76" s="6" t="n">
         <v>130</v>
@@ -2979,7 +3071,6 @@
         <v>-47.459</v>
       </c>
     </row>
-    <row r="126"/>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
         <is>
@@ -3130,14 +3221,22 @@
         <v>136.1385</v>
       </c>
     </row>
-    <row r="136"/>
-    <row r="137"/>
     <row r="138">
       <c r="A138" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B138" s="14" t="n"/>
+      <c r="C138" s="14" t="n"/>
+      <c r="D138" s="14" t="n"/>
+      <c r="E138" s="14" t="n"/>
+      <c r="F138" s="14" t="n"/>
+      <c r="G138" s="14" t="n"/>
+      <c r="H138" s="14" t="n"/>
+      <c r="I138" s="14" t="n"/>
+      <c r="J138" s="14" t="n"/>
+      <c r="K138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -3145,16 +3244,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B139" s="14" t="n"/>
+      <c r="C139" s="15" t="n"/>
       <c r="E139" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F139" s="14" t="n"/>
+      <c r="G139" s="15" t="n"/>
       <c r="I139" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J139" s="14" t="n"/>
+      <c r="K139" s="15" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="9" t="inlineStr">
@@ -4874,7 +4979,6 @@
         <v>-52.796</v>
       </c>
     </row>
-    <row r="225"/>
     <row r="226">
       <c r="A226" s="7" t="inlineStr">
         <is>
@@ -5073,14 +5177,33 @@
           <t>ExtraTrees — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -5088,16 +5211,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -6010,7 +6139,6 @@
         <v>1.56</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -6161,14 +6289,22 @@
         <v>33.834</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -6176,16 +6312,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -7106,7 +7248,6 @@
         <v>-14.759</v>
       </c>
     </row>
-    <row r="133"/>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
         <is>
@@ -7257,14 +7398,22 @@
         <v>25.6932</v>
       </c>
     </row>
-    <row r="143"/>
-    <row r="144"/>
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B145" s="14" t="n"/>
+      <c r="C145" s="14" t="n"/>
+      <c r="D145" s="14" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="14" t="n"/>
+      <c r="G145" s="14" t="n"/>
+      <c r="H145" s="14" t="n"/>
+      <c r="I145" s="14" t="n"/>
+      <c r="J145" s="14" t="n"/>
+      <c r="K145" s="15" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -7272,16 +7421,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B146" s="14" t="n"/>
+      <c r="C146" s="15" t="n"/>
       <c r="E146" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F146" s="14" t="n"/>
+      <c r="G146" s="15" t="n"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J146" s="14" t="n"/>
+      <c r="K146" s="15" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
@@ -9001,7 +9156,6 @@
         <v>-62.379</v>
       </c>
     </row>
-    <row r="232"/>
     <row r="233">
       <c r="A233" s="7" t="inlineStr">
         <is>
@@ -9200,14 +9354,33 @@
           <t>HistGradientBoosting — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -9215,16 +9388,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -10137,7 +10316,6 @@
         <v>-0.695</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -10288,14 +10466,22 @@
         <v>135.8788</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -10303,16 +10489,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -11223,7 +11415,6 @@
         <v>-49.127</v>
       </c>
     </row>
-    <row r="128"/>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
         <is>
@@ -11374,14 +11565,22 @@
         <v>173.2041</v>
       </c>
     </row>
-    <row r="138"/>
-    <row r="139"/>
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B140" s="14" t="n"/>
+      <c r="C140" s="14" t="n"/>
+      <c r="D140" s="14" t="n"/>
+      <c r="E140" s="14" t="n"/>
+      <c r="F140" s="14" t="n"/>
+      <c r="G140" s="14" t="n"/>
+      <c r="H140" s="14" t="n"/>
+      <c r="I140" s="14" t="n"/>
+      <c r="J140" s="14" t="n"/>
+      <c r="K140" s="15" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -11389,16 +11588,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B141" s="14" t="n"/>
+      <c r="C141" s="15" t="n"/>
       <c r="E141" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F141" s="14" t="n"/>
+      <c r="G141" s="15" t="n"/>
       <c r="I141" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J141" s="14" t="n"/>
+      <c r="K141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="9" t="inlineStr">
@@ -13118,7 +13323,6 @@
         <v>-29.954</v>
       </c>
     </row>
-    <row r="227"/>
     <row r="228">
       <c r="A228" s="7" t="inlineStr">
         <is>
@@ -13317,14 +13521,33 @@
           <t>Gaussian Process — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -13332,16 +13555,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -14254,7 +14483,6 @@
         <v>2.607</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -14405,14 +14633,22 @@
         <v>54.2098</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -14420,16 +14656,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -15340,7 +15582,6 @@
         <v>0.012</v>
       </c>
     </row>
-    <row r="128"/>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
         <is>
@@ -15491,14 +15732,22 @@
         <v>89.91849999999999</v>
       </c>
     </row>
-    <row r="138"/>
-    <row r="139"/>
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B140" s="14" t="n"/>
+      <c r="C140" s="14" t="n"/>
+      <c r="D140" s="14" t="n"/>
+      <c r="E140" s="14" t="n"/>
+      <c r="F140" s="14" t="n"/>
+      <c r="G140" s="14" t="n"/>
+      <c r="H140" s="14" t="n"/>
+      <c r="I140" s="14" t="n"/>
+      <c r="J140" s="14" t="n"/>
+      <c r="K140" s="15" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -15506,16 +15755,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B141" s="14" t="n"/>
+      <c r="C141" s="15" t="n"/>
       <c r="E141" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F141" s="14" t="n"/>
+      <c r="G141" s="15" t="n"/>
       <c r="I141" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J141" s="14" t="n"/>
+      <c r="K141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="9" t="inlineStr">
@@ -17235,7 +17490,6 @@
         <v>-57.127</v>
       </c>
     </row>
-    <row r="227"/>
     <row r="228">
       <c r="A228" s="7" t="inlineStr">
         <is>
@@ -17434,14 +17688,33 @@
           <t>Stacked Ensemble — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -17449,16 +17722,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -18371,7 +18650,6 @@
         <v>0.969</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -18522,14 +18800,22 @@
         <v>65.34910000000001</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -18537,16 +18823,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -19457,7 +19749,6 @@
         <v>5.001</v>
       </c>
     </row>
-    <row r="128"/>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
         <is>
@@ -19608,14 +19899,22 @@
         <v>58.9637</v>
       </c>
     </row>
-    <row r="138"/>
-    <row r="139"/>
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B140" s="14" t="n"/>
+      <c r="C140" s="14" t="n"/>
+      <c r="D140" s="14" t="n"/>
+      <c r="E140" s="14" t="n"/>
+      <c r="F140" s="14" t="n"/>
+      <c r="G140" s="14" t="n"/>
+      <c r="H140" s="14" t="n"/>
+      <c r="I140" s="14" t="n"/>
+      <c r="J140" s="14" t="n"/>
+      <c r="K140" s="15" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -19623,16 +19922,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B141" s="14" t="n"/>
+      <c r="C141" s="15" t="n"/>
       <c r="E141" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F141" s="14" t="n"/>
+      <c r="G141" s="15" t="n"/>
       <c r="I141" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J141" s="14" t="n"/>
+      <c r="K141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="9" t="inlineStr">
@@ -21352,7 +21657,6 @@
         <v>-53.507</v>
       </c>
     </row>
-    <row r="227"/>
     <row r="228">
       <c r="A228" s="7" t="inlineStr">
         <is>
@@ -21551,14 +21855,33 @@
           <t>MLP (ANN) — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -21566,16 +21889,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -22488,7 +22817,6 @@
         <v>0.522</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -22639,14 +22967,22 @@
         <v>68.1644</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -22654,16 +22990,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -23570,7 +23912,6 @@
         <v>-46.518</v>
       </c>
     </row>
-    <row r="126"/>
     <row r="127">
       <c r="A127" s="7" t="inlineStr">
         <is>
@@ -23721,14 +24062,22 @@
         <v>132.7059</v>
       </c>
     </row>
-    <row r="136"/>
-    <row r="137"/>
     <row r="138">
       <c r="A138" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B138" s="14" t="n"/>
+      <c r="C138" s="14" t="n"/>
+      <c r="D138" s="14" t="n"/>
+      <c r="E138" s="14" t="n"/>
+      <c r="F138" s="14" t="n"/>
+      <c r="G138" s="14" t="n"/>
+      <c r="H138" s="14" t="n"/>
+      <c r="I138" s="14" t="n"/>
+      <c r="J138" s="14" t="n"/>
+      <c r="K138" s="15" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -23736,16 +24085,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B139" s="14" t="n"/>
+      <c r="C139" s="15" t="n"/>
       <c r="E139" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F139" s="14" t="n"/>
+      <c r="G139" s="15" t="n"/>
       <c r="I139" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J139" s="14" t="n"/>
+      <c r="K139" s="15" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="9" t="inlineStr">
@@ -25465,7 +25820,6 @@
         <v>-132.779</v>
       </c>
     </row>
-    <row r="225"/>
     <row r="226">
       <c r="A226" s="7" t="inlineStr">
         <is>
@@ -25664,14 +26018,33 @@
           <t>BoostStack — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -25679,16 +26052,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -26601,7 +26980,6 @@
         <v>-7.496</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -26752,14 +27130,22 @@
         <v>37.1935</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -26767,16 +27153,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -27697,7 +28089,6 @@
         <v>-5.022</v>
       </c>
     </row>
-    <row r="133"/>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
         <is>
@@ -27848,14 +28239,22 @@
         <v>30.5827</v>
       </c>
     </row>
-    <row r="143"/>
-    <row r="144"/>
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B145" s="14" t="n"/>
+      <c r="C145" s="14" t="n"/>
+      <c r="D145" s="14" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="14" t="n"/>
+      <c r="G145" s="14" t="n"/>
+      <c r="H145" s="14" t="n"/>
+      <c r="I145" s="14" t="n"/>
+      <c r="J145" s="14" t="n"/>
+      <c r="K145" s="15" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -27863,16 +28262,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B146" s="14" t="n"/>
+      <c r="C146" s="15" t="n"/>
       <c r="E146" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F146" s="14" t="n"/>
+      <c r="G146" s="15" t="n"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J146" s="14" t="n"/>
+      <c r="K146" s="15" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
@@ -29592,7 +29997,6 @@
         <v>-71.938</v>
       </c>
     </row>
-    <row r="232"/>
     <row r="233">
       <c r="A233" s="7" t="inlineStr">
         <is>
@@ -29791,14 +30195,33 @@
           <t>GB_seed_ensemble — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -29806,16 +30229,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -30728,7 +31157,6 @@
         <v>1.191</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -30879,14 +31307,22 @@
         <v>24.41</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -30894,16 +31330,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -31824,7 +32266,6 @@
         <v>-0.231</v>
       </c>
     </row>
-    <row r="133"/>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
         <is>
@@ -31975,14 +32416,22 @@
         <v>33.27</v>
       </c>
     </row>
-    <row r="143"/>
-    <row r="144"/>
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B145" s="14" t="n"/>
+      <c r="C145" s="14" t="n"/>
+      <c r="D145" s="14" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="14" t="n"/>
+      <c r="G145" s="14" t="n"/>
+      <c r="H145" s="14" t="n"/>
+      <c r="I145" s="14" t="n"/>
+      <c r="J145" s="14" t="n"/>
+      <c r="K145" s="15" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -31990,16 +32439,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B146" s="14" t="n"/>
+      <c r="C146" s="15" t="n"/>
       <c r="E146" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F146" s="14" t="n"/>
+      <c r="G146" s="15" t="n"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J146" s="14" t="n"/>
+      <c r="K146" s="15" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
@@ -33719,7 +34174,6 @@
         <v>-68.55200000000001</v>
       </c>
     </row>
-    <row r="232"/>
     <row r="233">
       <c r="A233" s="7" t="inlineStr">
         <is>
@@ -33909,6 +34363,7 @@
           <t>METHODOLOGY</t>
         </is>
       </c>
+      <c r="B1" s="15" t="n"/>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
@@ -34081,6 +34536,31 @@
           <t>MODEL PERFORMANCE METRICS SUMMARY — SLUMP (CV-averaged)</t>
         </is>
       </c>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="14" t="n"/>
+      <c r="L1" s="14" t="n"/>
+      <c r="M1" s="14" t="n"/>
+      <c r="N1" s="14" t="n"/>
+      <c r="O1" s="14" t="n"/>
+      <c r="P1" s="14" t="n"/>
+      <c r="Q1" s="14" t="n"/>
+      <c r="R1" s="14" t="n"/>
+      <c r="S1" s="14" t="n"/>
+      <c r="T1" s="14" t="n"/>
+      <c r="U1" s="14" t="n"/>
+      <c r="V1" s="14" t="n"/>
+      <c r="W1" s="14" t="n"/>
+      <c r="X1" s="14" t="n"/>
+      <c r="Y1" s="14" t="n"/>
+      <c r="Z1" s="15" t="n"/>
     </row>
     <row r="2"/>
     <row r="3">
@@ -34089,6 +34569,31 @@
           <t>REGIME 1 — Random KFold (5 folds × 5 repeats, industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="14" t="n"/>
+      <c r="L3" s="14" t="n"/>
+      <c r="M3" s="14" t="n"/>
+      <c r="N3" s="14" t="n"/>
+      <c r="O3" s="14" t="n"/>
+      <c r="P3" s="14" t="n"/>
+      <c r="Q3" s="14" t="n"/>
+      <c r="R3" s="14" t="n"/>
+      <c r="S3" s="14" t="n"/>
+      <c r="T3" s="14" t="n"/>
+      <c r="U3" s="14" t="n"/>
+      <c r="V3" s="14" t="n"/>
+      <c r="W3" s="14" t="n"/>
+      <c r="X3" s="14" t="n"/>
+      <c r="Y3" s="14" t="n"/>
+      <c r="Z3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -34101,16 +34606,37 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="14" t="n"/>
+      <c r="E4" s="14" t="n"/>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="14" t="n"/>
+      <c r="H4" s="14" t="n"/>
+      <c r="I4" s="15" t="n"/>
       <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="K4" s="14" t="n"/>
+      <c r="L4" s="14" t="n"/>
+      <c r="M4" s="14" t="n"/>
+      <c r="N4" s="14" t="n"/>
+      <c r="O4" s="14" t="n"/>
+      <c r="P4" s="14" t="n"/>
+      <c r="Q4" s="15" t="n"/>
       <c r="R4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="S4" s="14" t="n"/>
+      <c r="T4" s="14" t="n"/>
+      <c r="U4" s="14" t="n"/>
+      <c r="V4" s="14" t="n"/>
+      <c r="W4" s="14" t="n"/>
+      <c r="X4" s="14" t="n"/>
+      <c r="Y4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="9" t="inlineStr">
@@ -35426,6 +35952,31 @@
           <t>REGIME 2 — GroupKFold strict (no mix-design leakage, honest)</t>
         </is>
       </c>
+      <c r="B22" s="14" t="n"/>
+      <c r="C22" s="14" t="n"/>
+      <c r="D22" s="14" t="n"/>
+      <c r="E22" s="14" t="n"/>
+      <c r="F22" s="14" t="n"/>
+      <c r="G22" s="14" t="n"/>
+      <c r="H22" s="14" t="n"/>
+      <c r="I22" s="14" t="n"/>
+      <c r="J22" s="14" t="n"/>
+      <c r="K22" s="14" t="n"/>
+      <c r="L22" s="14" t="n"/>
+      <c r="M22" s="14" t="n"/>
+      <c r="N22" s="14" t="n"/>
+      <c r="O22" s="14" t="n"/>
+      <c r="P22" s="14" t="n"/>
+      <c r="Q22" s="14" t="n"/>
+      <c r="R22" s="14" t="n"/>
+      <c r="S22" s="14" t="n"/>
+      <c r="T22" s="14" t="n"/>
+      <c r="U22" s="14" t="n"/>
+      <c r="V22" s="14" t="n"/>
+      <c r="W22" s="14" t="n"/>
+      <c r="X22" s="14" t="n"/>
+      <c r="Y22" s="14" t="n"/>
+      <c r="Z22" s="15" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -35438,16 +35989,37 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="14" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="14" t="n"/>
+      <c r="G23" s="14" t="n"/>
+      <c r="H23" s="14" t="n"/>
+      <c r="I23" s="15" t="n"/>
       <c r="J23" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="K23" s="14" t="n"/>
+      <c r="L23" s="14" t="n"/>
+      <c r="M23" s="14" t="n"/>
+      <c r="N23" s="14" t="n"/>
+      <c r="O23" s="14" t="n"/>
+      <c r="P23" s="14" t="n"/>
+      <c r="Q23" s="15" t="n"/>
       <c r="R23" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="S23" s="14" t="n"/>
+      <c r="T23" s="14" t="n"/>
+      <c r="U23" s="14" t="n"/>
+      <c r="V23" s="14" t="n"/>
+      <c r="W23" s="14" t="n"/>
+      <c r="X23" s="14" t="n"/>
+      <c r="Y23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="9" t="inlineStr">
@@ -36763,6 +37335,31 @@
           <t>REGIME 3 — LOOCV (Leave-One-Out, report-side high-R² protocol)</t>
         </is>
       </c>
+      <c r="B41" s="14" t="n"/>
+      <c r="C41" s="14" t="n"/>
+      <c r="D41" s="14" t="n"/>
+      <c r="E41" s="14" t="n"/>
+      <c r="F41" s="14" t="n"/>
+      <c r="G41" s="14" t="n"/>
+      <c r="H41" s="14" t="n"/>
+      <c r="I41" s="14" t="n"/>
+      <c r="J41" s="14" t="n"/>
+      <c r="K41" s="14" t="n"/>
+      <c r="L41" s="14" t="n"/>
+      <c r="M41" s="14" t="n"/>
+      <c r="N41" s="14" t="n"/>
+      <c r="O41" s="14" t="n"/>
+      <c r="P41" s="14" t="n"/>
+      <c r="Q41" s="14" t="n"/>
+      <c r="R41" s="14" t="n"/>
+      <c r="S41" s="14" t="n"/>
+      <c r="T41" s="14" t="n"/>
+      <c r="U41" s="14" t="n"/>
+      <c r="V41" s="14" t="n"/>
+      <c r="W41" s="14" t="n"/>
+      <c r="X41" s="14" t="n"/>
+      <c r="Y41" s="14" t="n"/>
+      <c r="Z41" s="15" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -36775,16 +37372,37 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="14" t="n"/>
+      <c r="E42" s="14" t="n"/>
+      <c r="F42" s="14" t="n"/>
+      <c r="G42" s="14" t="n"/>
+      <c r="H42" s="14" t="n"/>
+      <c r="I42" s="15" t="n"/>
       <c r="J42" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="K42" s="14" t="n"/>
+      <c r="L42" s="14" t="n"/>
+      <c r="M42" s="14" t="n"/>
+      <c r="N42" s="14" t="n"/>
+      <c r="O42" s="14" t="n"/>
+      <c r="P42" s="14" t="n"/>
+      <c r="Q42" s="15" t="n"/>
       <c r="R42" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="S42" s="14" t="n"/>
+      <c r="T42" s="14" t="n"/>
+      <c r="U42" s="14" t="n"/>
+      <c r="V42" s="14" t="n"/>
+      <c r="W42" s="14" t="n"/>
+      <c r="X42" s="14" t="n"/>
+      <c r="Y42" s="15" t="n"/>
     </row>
     <row r="43">
       <c r="B43" s="9" t="inlineStr">
@@ -37941,34 +38559,78 @@
           <t>BoostStack</t>
         </is>
       </c>
-      <c r="B57" s="12" t="n"/>
-      <c r="C57" s="12" t="n"/>
-      <c r="D57" s="12" t="n"/>
-      <c r="E57" s="12" t="n">
-        <v>0.9994</v>
-      </c>
-      <c r="F57" s="12" t="n"/>
-      <c r="G57" s="12" t="n"/>
-      <c r="H57" s="12" t="n"/>
-      <c r="I57" s="12" t="n"/>
-      <c r="J57" s="12" t="n"/>
-      <c r="K57" s="12" t="n"/>
-      <c r="L57" s="12" t="n"/>
-      <c r="M57" s="12" t="n"/>
-      <c r="N57" s="12" t="n"/>
-      <c r="O57" s="12" t="n"/>
-      <c r="P57" s="12" t="n"/>
-      <c r="Q57" s="12" t="n"/>
-      <c r="R57" s="12" t="n"/>
-      <c r="S57" s="12" t="n"/>
-      <c r="T57" s="12" t="n"/>
-      <c r="U57" s="12" t="n">
-        <v>0.9448</v>
-      </c>
-      <c r="V57" s="12" t="n"/>
-      <c r="W57" s="12" t="n"/>
-      <c r="X57" s="12" t="n"/>
-      <c r="Y57" s="12" t="n"/>
+      <c r="B57" s="16" t="n">
+        <v>4.7124</v>
+      </c>
+      <c r="C57" s="16" t="n">
+        <v>51.37</v>
+      </c>
+      <c r="D57" s="16" t="n">
+        <v>7.1673</v>
+      </c>
+      <c r="E57" s="16" t="n">
+        <v>0.9971</v>
+      </c>
+      <c r="F57" s="16" t="n">
+        <v>0.9442</v>
+      </c>
+      <c r="G57" s="16" t="n">
+        <v>0.0351</v>
+      </c>
+      <c r="H57" s="16" t="n">
+        <v>99.7146</v>
+      </c>
+      <c r="I57" s="16" t="n">
+        <v>7.124</v>
+      </c>
+      <c r="J57" s="16" t="n">
+        <v>26.3888</v>
+      </c>
+      <c r="K57" s="16" t="n">
+        <v>1388.9275</v>
+      </c>
+      <c r="L57" s="16" t="n">
+        <v>37.2683</v>
+      </c>
+      <c r="M57" s="16" t="n">
+        <v>0.8934</v>
+      </c>
+      <c r="N57" s="16" t="n">
+        <v>0.6271</v>
+      </c>
+      <c r="O57" s="16" t="n">
+        <v>0.2371</v>
+      </c>
+      <c r="P57" s="16" t="n">
+        <v>89.355</v>
+      </c>
+      <c r="Q57" s="16" t="n">
+        <v>37.2434</v>
+      </c>
+      <c r="R57" s="16" t="n">
+        <v>21.4866</v>
+      </c>
+      <c r="S57" s="16" t="n">
+        <v>996.004</v>
+      </c>
+      <c r="T57" s="16" t="n">
+        <v>31.5595</v>
+      </c>
+      <c r="U57" s="16" t="n">
+        <v>0.9403</v>
+      </c>
+      <c r="V57" s="16" t="n">
+        <v>0.7352</v>
+      </c>
+      <c r="W57" s="16" t="n">
+        <v>0.1977</v>
+      </c>
+      <c r="X57" s="16" t="n">
+        <v>94.03830000000001</v>
+      </c>
+      <c r="Y57" s="16" t="n">
+        <v>31.5493</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
@@ -37976,34 +38638,78 @@
           <t>GB_seed_ensemble</t>
         </is>
       </c>
-      <c r="B58" s="11" t="n"/>
-      <c r="C58" s="11" t="n"/>
-      <c r="D58" s="11" t="n"/>
-      <c r="E58" s="11" t="n">
-        <v>0.9987</v>
-      </c>
-      <c r="F58" s="11" t="n"/>
-      <c r="G58" s="11" t="n"/>
-      <c r="H58" s="11" t="n"/>
-      <c r="I58" s="11" t="n"/>
-      <c r="J58" s="11" t="n"/>
-      <c r="K58" s="11" t="n"/>
-      <c r="L58" s="11" t="n"/>
-      <c r="M58" s="11" t="n"/>
-      <c r="N58" s="11" t="n"/>
-      <c r="O58" s="11" t="n"/>
-      <c r="P58" s="11" t="n"/>
-      <c r="Q58" s="11" t="n"/>
-      <c r="R58" s="11" t="n"/>
-      <c r="S58" s="11" t="n"/>
-      <c r="T58" s="11" t="n"/>
-      <c r="U58" s="11" t="n">
-        <v>0.9519</v>
-      </c>
-      <c r="V58" s="11" t="n"/>
-      <c r="W58" s="11" t="n"/>
-      <c r="X58" s="11" t="n"/>
-      <c r="Y58" s="11" t="n"/>
+      <c r="B58" s="17" t="n">
+        <v>1.2133</v>
+      </c>
+      <c r="C58" s="17" t="n">
+        <v>8.980700000000001</v>
+      </c>
+      <c r="D58" s="17" t="n">
+        <v>2.9968</v>
+      </c>
+      <c r="E58" s="17" t="n">
+        <v>0.9995000000000001</v>
+      </c>
+      <c r="F58" s="17" t="n">
+        <v>0.9856</v>
+      </c>
+      <c r="G58" s="17" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="H58" s="17" t="n">
+        <v>99.9495</v>
+      </c>
+      <c r="I58" s="17" t="n">
+        <v>2.9967</v>
+      </c>
+      <c r="J58" s="17" t="n">
+        <v>24.2944</v>
+      </c>
+      <c r="K58" s="17" t="n">
+        <v>1293.7505</v>
+      </c>
+      <c r="L58" s="17" t="n">
+        <v>35.9687</v>
+      </c>
+      <c r="M58" s="17" t="n">
+        <v>0.9006999999999999</v>
+      </c>
+      <c r="N58" s="17" t="n">
+        <v>0.6567</v>
+      </c>
+      <c r="O58" s="17" t="n">
+        <v>0.2193</v>
+      </c>
+      <c r="P58" s="17" t="n">
+        <v>90.0767</v>
+      </c>
+      <c r="Q58" s="17" t="n">
+        <v>35.9588</v>
+      </c>
+      <c r="R58" s="17" t="n">
+        <v>19.0842</v>
+      </c>
+      <c r="S58" s="17" t="n">
+        <v>774.4399</v>
+      </c>
+      <c r="T58" s="17" t="n">
+        <v>27.8288</v>
+      </c>
+      <c r="U58" s="17" t="n">
+        <v>0.9536</v>
+      </c>
+      <c r="V58" s="17" t="n">
+        <v>0.7648</v>
+      </c>
+      <c r="W58" s="17" t="n">
+        <v>0.1776</v>
+      </c>
+      <c r="X58" s="17" t="n">
+        <v>95.3644</v>
+      </c>
+      <c r="Y58" s="17" t="n">
+        <v>27.82</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -38053,14 +38759,33 @@
           <t>Linear Regression — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -38068,16 +38793,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -38990,7 +39721,6 @@
         <v>57.443</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -39141,14 +39871,22 @@
         <v>50.9809</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -39156,16 +39894,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -40086,7 +40830,6 @@
         <v>-98.25</v>
       </c>
     </row>
-    <row r="133"/>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
         <is>
@@ -40237,14 +40980,22 @@
         <v>88.7732</v>
       </c>
     </row>
-    <row r="143"/>
-    <row r="144"/>
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B145" s="14" t="n"/>
+      <c r="C145" s="14" t="n"/>
+      <c r="D145" s="14" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="14" t="n"/>
+      <c r="G145" s="14" t="n"/>
+      <c r="H145" s="14" t="n"/>
+      <c r="I145" s="14" t="n"/>
+      <c r="J145" s="14" t="n"/>
+      <c r="K145" s="15" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -40252,16 +41003,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B146" s="14" t="n"/>
+      <c r="C146" s="15" t="n"/>
       <c r="E146" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F146" s="14" t="n"/>
+      <c r="G146" s="15" t="n"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J146" s="14" t="n"/>
+      <c r="K146" s="15" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
@@ -41981,7 +42738,6 @@
         <v>-126.266</v>
       </c>
     </row>
-    <row r="232"/>
     <row r="233">
       <c r="A233" s="7" t="inlineStr">
         <is>
@@ -42180,14 +42936,33 @@
           <t>Random Forest — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -42195,16 +42970,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -43117,7 +43898,6 @@
         <v>8.914</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -43268,14 +44048,22 @@
         <v>42.0112</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -43283,16 +44071,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -44213,7 +45007,6 @@
         <v>-26.704</v>
       </c>
     </row>
-    <row r="133"/>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
         <is>
@@ -44364,14 +45157,22 @@
         <v>30.3934</v>
       </c>
     </row>
-    <row r="143"/>
-    <row r="144"/>
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B145" s="14" t="n"/>
+      <c r="C145" s="14" t="n"/>
+      <c r="D145" s="14" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="14" t="n"/>
+      <c r="G145" s="14" t="n"/>
+      <c r="H145" s="14" t="n"/>
+      <c r="I145" s="14" t="n"/>
+      <c r="J145" s="14" t="n"/>
+      <c r="K145" s="15" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -44379,16 +45180,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B146" s="14" t="n"/>
+      <c r="C146" s="15" t="n"/>
       <c r="E146" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F146" s="14" t="n"/>
+      <c r="G146" s="15" t="n"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J146" s="14" t="n"/>
+      <c r="K146" s="15" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
@@ -46108,7 +46915,6 @@
         <v>-61.766</v>
       </c>
     </row>
-    <row r="232"/>
     <row r="233">
       <c r="A233" s="7" t="inlineStr">
         <is>
@@ -46307,14 +47113,33 @@
           <t>Gradient Boosting — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -46322,16 +47147,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -47244,7 +48075,6 @@
         <v>0.874</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -47395,14 +48225,22 @@
         <v>26.8788</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -47410,16 +48248,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -48340,7 +49184,6 @@
         <v>0.202</v>
       </c>
     </row>
-    <row r="133"/>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
         <is>
@@ -48491,14 +49334,22 @@
         <v>32.9876</v>
       </c>
     </row>
-    <row r="143"/>
-    <row r="144"/>
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B145" s="14" t="n"/>
+      <c r="C145" s="14" t="n"/>
+      <c r="D145" s="14" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="14" t="n"/>
+      <c r="G145" s="14" t="n"/>
+      <c r="H145" s="14" t="n"/>
+      <c r="I145" s="14" t="n"/>
+      <c r="J145" s="14" t="n"/>
+      <c r="K145" s="15" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -48506,16 +49357,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B146" s="14" t="n"/>
+      <c r="C146" s="15" t="n"/>
       <c r="E146" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F146" s="14" t="n"/>
+      <c r="G146" s="15" t="n"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J146" s="14" t="n"/>
+      <c r="K146" s="15" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
@@ -50235,7 +51092,6 @@
         <v>-79.69199999999999</v>
       </c>
     </row>
-    <row r="232"/>
     <row r="233">
       <c r="A233" s="7" t="inlineStr">
         <is>
@@ -50434,14 +51290,33 @@
           <t>AdaBoost — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -50449,16 +51324,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -51371,7 +52252,6 @@
         <v>-4</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -51522,14 +52402,22 @@
         <v>38.2844</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -51537,16 +52425,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -52467,7 +53361,6 @@
         <v>-2.2</v>
       </c>
     </row>
-    <row r="133"/>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
         <is>
@@ -52618,14 +53511,22 @@
         <v>33.9969</v>
       </c>
     </row>
-    <row r="143"/>
-    <row r="144"/>
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B145" s="14" t="n"/>
+      <c r="C145" s="14" t="n"/>
+      <c r="D145" s="14" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="14" t="n"/>
+      <c r="G145" s="14" t="n"/>
+      <c r="H145" s="14" t="n"/>
+      <c r="I145" s="14" t="n"/>
+      <c r="J145" s="14" t="n"/>
+      <c r="K145" s="15" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -52633,16 +53534,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B146" s="14" t="n"/>
+      <c r="C146" s="15" t="n"/>
       <c r="E146" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F146" s="14" t="n"/>
+      <c r="G146" s="15" t="n"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J146" s="14" t="n"/>
+      <c r="K146" s="15" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
@@ -54362,7 +55269,6 @@
         <v>-66.27800000000001</v>
       </c>
     </row>
-    <row r="232"/>
     <row r="233">
       <c r="A233" s="7" t="inlineStr">
         <is>
@@ -54561,14 +55467,33 @@
           <t>CatBoost — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -54576,16 +55501,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -54671,7 +55602,7 @@
         <v>173</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E7" s="6" t="n">
         <v>220</v>
@@ -54700,7 +55631,7 @@
         <v>275</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>130</v>
@@ -54758,7 +55689,7 @@
         <v>75</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>145</v>
@@ -54903,7 +55834,7 @@
         <v>255</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E15" s="6" t="n">
         <v>43</v>
@@ -54932,7 +55863,7 @@
         <v>285</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E16" s="4" t="n">
         <v>620</v>
@@ -55079,7 +56010,7 @@
         <v>220</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I22" s="4" t="n">
         <v>200</v>
@@ -55099,7 +56030,7 @@
         <v>580</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -55110,7 +56041,7 @@
         <v>165</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -55121,7 +56052,7 @@
         <v>120</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -55132,7 +56063,7 @@
         <v>190</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -55143,7 +56074,7 @@
         <v>130</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -55187,7 +56118,7 @@
         <v>155</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -55209,7 +56140,7 @@
         <v>205</v>
       </c>
       <c r="C33" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -55231,7 +56162,7 @@
         <v>144</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -55264,7 +56195,7 @@
         <v>185</v>
       </c>
       <c r="C38" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -55275,7 +56206,7 @@
         <v>225</v>
       </c>
       <c r="C39" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -55297,7 +56228,7 @@
         <v>70</v>
       </c>
       <c r="C41" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -55319,7 +56250,7 @@
         <v>195</v>
       </c>
       <c r="C43" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -55330,7 +56261,7 @@
         <v>175</v>
       </c>
       <c r="C44" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -55341,7 +56272,7 @@
         <v>200</v>
       </c>
       <c r="C45" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
@@ -55407,7 +56338,7 @@
         <v>86</v>
       </c>
       <c r="C51" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -55429,7 +56360,7 @@
         <v>190</v>
       </c>
       <c r="C53" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54">
@@ -55451,7 +56382,7 @@
         <v>62</v>
       </c>
       <c r="C55" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -55462,7 +56393,7 @@
         <v>650</v>
       </c>
       <c r="C56" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57">
@@ -55473,7 +56404,7 @@
         <v>150</v>
       </c>
       <c r="C57" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
@@ -55484,7 +56415,7 @@
         <v>160</v>
       </c>
       <c r="C58" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
@@ -55495,10 +56426,9 @@
         <v>210</v>
       </c>
       <c r="C59" s="6" t="n">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="60"/>
+        <v>0</v>
+      </c>
+    </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -55649,14 +56579,22 @@
         <v>32.3844</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -55664,16 +56602,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -55759,7 +56703,7 @@
         <v>160</v>
       </c>
       <c r="C76" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E76" s="6" t="n">
         <v>210</v>
@@ -55817,7 +56761,7 @@
         <v>180</v>
       </c>
       <c r="C78" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E78" s="6" t="n">
         <v>155</v>
@@ -55875,7 +56819,7 @@
         <v>130</v>
       </c>
       <c r="C80" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E80" s="6" t="n">
         <v>170</v>
@@ -55933,7 +56877,7 @@
         <v>190</v>
       </c>
       <c r="C82" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E82" s="6" t="n">
         <v>185</v>
@@ -55991,7 +56935,7 @@
         <v>195</v>
       </c>
       <c r="C84" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E84" s="6" t="n">
         <v>227</v>
@@ -56049,7 +56993,7 @@
         <v>205</v>
       </c>
       <c r="C86" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E86" s="6" t="n">
         <v>200</v>
@@ -56107,7 +57051,7 @@
         <v>220</v>
       </c>
       <c r="C88" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E88" s="6" t="n">
         <v>220</v>
@@ -56136,7 +57080,7 @@
         <v>120</v>
       </c>
       <c r="C89" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I89" s="4" t="n">
         <v>32</v>
@@ -56156,7 +57100,7 @@
         <v>124</v>
       </c>
       <c r="C90" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I90" s="6" t="n">
         <v>60</v>
@@ -56196,7 +57140,7 @@
         <v>140</v>
       </c>
       <c r="C92" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93">
@@ -56218,7 +57162,7 @@
         <v>620</v>
       </c>
       <c r="C94" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95">
@@ -56240,7 +57184,7 @@
         <v>550</v>
       </c>
       <c r="C96" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="97">
@@ -56262,7 +57206,7 @@
         <v>620</v>
       </c>
       <c r="C98" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99">
@@ -56284,7 +57228,7 @@
         <v>200</v>
       </c>
       <c r="C100" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101">
@@ -56306,7 +57250,7 @@
         <v>290</v>
       </c>
       <c r="C102" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103">
@@ -56328,7 +57272,7 @@
         <v>275</v>
       </c>
       <c r="C104" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105">
@@ -56350,7 +57294,7 @@
         <v>185</v>
       </c>
       <c r="C106" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107">
@@ -56361,7 +57305,7 @@
         <v>130</v>
       </c>
       <c r="C107" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108">
@@ -56416,7 +57360,7 @@
         <v>173</v>
       </c>
       <c r="C112" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -56438,7 +57382,7 @@
         <v>145</v>
       </c>
       <c r="C114" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115">
@@ -56471,7 +57415,7 @@
         <v>75</v>
       </c>
       <c r="C117" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118">
@@ -56504,7 +57448,7 @@
         <v>40</v>
       </c>
       <c r="C120" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="121">
@@ -56537,7 +57481,7 @@
         <v>160</v>
       </c>
       <c r="C123" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="124">
@@ -56559,7 +57503,7 @@
         <v>50</v>
       </c>
       <c r="C125" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126">
@@ -56584,7 +57528,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128"/>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
         <is>
@@ -56735,14 +57678,22 @@
         <v>59.2266</v>
       </c>
     </row>
-    <row r="138"/>
-    <row r="139"/>
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B140" s="14" t="n"/>
+      <c r="C140" s="14" t="n"/>
+      <c r="D140" s="14" t="n"/>
+      <c r="E140" s="14" t="n"/>
+      <c r="F140" s="14" t="n"/>
+      <c r="G140" s="14" t="n"/>
+      <c r="H140" s="14" t="n"/>
+      <c r="I140" s="14" t="n"/>
+      <c r="J140" s="14" t="n"/>
+      <c r="K140" s="15" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -56750,16 +57701,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B141" s="14" t="n"/>
+      <c r="C141" s="15" t="n"/>
       <c r="E141" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F141" s="14" t="n"/>
+      <c r="G141" s="15" t="n"/>
       <c r="I141" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J141" s="14" t="n"/>
+      <c r="K141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="9" t="inlineStr">
@@ -56816,7 +57773,7 @@
         <v>62</v>
       </c>
       <c r="C143" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E143" s="4" t="n">
         <v>220</v>
@@ -56990,7 +57947,7 @@
         <v>190</v>
       </c>
       <c r="C149" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E149" s="4" t="n">
         <v>175</v>
@@ -57019,7 +57976,7 @@
         <v>265</v>
       </c>
       <c r="C150" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E150" s="6" t="n">
         <v>215</v>
@@ -57193,7 +58150,7 @@
         <v>165</v>
       </c>
       <c r="C156" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E156" s="6" t="n">
         <v>195</v>
@@ -57569,7 +58526,7 @@
         <v>180</v>
       </c>
       <c r="C173" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I173" s="4" t="n">
         <v>124</v>
@@ -57589,7 +58546,7 @@
         <v>130</v>
       </c>
       <c r="C174" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I174" s="6" t="n">
         <v>130</v>
@@ -57649,7 +58606,7 @@
         <v>176</v>
       </c>
       <c r="C177" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I177" s="4" t="n">
         <v>620</v>
@@ -57749,7 +58706,7 @@
         <v>220</v>
       </c>
       <c r="C182" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I182" s="6" t="n">
         <v>580</v>
@@ -57769,7 +58726,7 @@
         <v>200</v>
       </c>
       <c r="C183" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I183" s="4" t="n">
         <v>175</v>
@@ -57789,7 +58746,7 @@
         <v>86</v>
       </c>
       <c r="C184" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I184" s="6" t="n">
         <v>200</v>
@@ -57829,7 +58786,7 @@
         <v>165</v>
       </c>
       <c r="C186" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I186" s="6" t="n">
         <v>290</v>
@@ -57849,7 +58806,7 @@
         <v>185</v>
       </c>
       <c r="C187" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I187" s="4" t="n">
         <v>285</v>
@@ -57909,7 +58866,7 @@
         <v>155</v>
       </c>
       <c r="C190" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I190" s="6" t="n">
         <v>220</v>
@@ -57929,7 +58886,7 @@
         <v>220</v>
       </c>
       <c r="C191" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I191" s="4" t="n">
         <v>185</v>
@@ -58009,7 +58966,7 @@
         <v>32</v>
       </c>
       <c r="C195" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I195" s="4" t="n">
         <v>150</v>
@@ -58049,7 +59006,7 @@
         <v>70</v>
       </c>
       <c r="C197" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I197" s="4" t="n">
         <v>227</v>
@@ -58069,7 +59026,7 @@
         <v>210</v>
       </c>
       <c r="C198" s="6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I198" s="6" t="n">
         <v>223</v>
@@ -58209,7 +59166,7 @@
         <v>210</v>
       </c>
       <c r="C205" s="4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I205" s="4" t="n">
         <v>80</v>
@@ -58479,7 +59436,6 @@
         <v>-49.702</v>
       </c>
     </row>
-    <row r="227"/>
     <row r="228">
       <c r="A228" s="7" t="inlineStr">
         <is>
@@ -58678,14 +59634,33 @@
           <t>LightGBM — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -58693,16 +59668,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -59615,7 +60596,6 @@
         <v>-0.151</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -59766,14 +60746,22 @@
         <v>44.3775</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -59781,16 +60769,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -60701,7 +61695,6 @@
         <v>0.679</v>
       </c>
     </row>
-    <row r="128"/>
     <row r="129">
       <c r="A129" s="7" t="inlineStr">
         <is>
@@ -60852,14 +61845,22 @@
         <v>44.6089</v>
       </c>
     </row>
-    <row r="138"/>
-    <row r="139"/>
     <row r="140">
       <c r="A140" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B140" s="14" t="n"/>
+      <c r="C140" s="14" t="n"/>
+      <c r="D140" s="14" t="n"/>
+      <c r="E140" s="14" t="n"/>
+      <c r="F140" s="14" t="n"/>
+      <c r="G140" s="14" t="n"/>
+      <c r="H140" s="14" t="n"/>
+      <c r="I140" s="14" t="n"/>
+      <c r="J140" s="14" t="n"/>
+      <c r="K140" s="15" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -60867,16 +61868,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B141" s="14" t="n"/>
+      <c r="C141" s="15" t="n"/>
       <c r="E141" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F141" s="14" t="n"/>
+      <c r="G141" s="15" t="n"/>
       <c r="I141" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J141" s="14" t="n"/>
+      <c r="K141" s="15" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="9" t="inlineStr">
@@ -62596,7 +63603,6 @@
         <v>-47.942</v>
       </c>
     </row>
-    <row r="227"/>
     <row r="228">
       <c r="A228" s="7" t="inlineStr">
         <is>
@@ -62795,14 +63801,33 @@
           <t>XGBoost — Predictions vs Actual (representative fold per regime)</t>
         </is>
       </c>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
+      <c r="G1" s="14" t="n"/>
+      <c r="H1" s="14" t="n"/>
+      <c r="I1" s="14" t="n"/>
+      <c r="J1" s="14" t="n"/>
+      <c r="K1" s="15" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Random KFold (industry-comparable)</t>
         </is>
       </c>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -62810,16 +63835,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B4" s="14" t="n"/>
+      <c r="C4" s="15" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="15" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="15" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -63732,7 +64763,6 @@
         <v>0.283</v>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
@@ -63883,14 +64913,22 @@
         <v>35.3499</v>
       </c>
     </row>
-    <row r="70"/>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
         <is>
           <t>GroupKFold strict (honest)</t>
         </is>
       </c>
+      <c r="B72" s="14" t="n"/>
+      <c r="C72" s="14" t="n"/>
+      <c r="D72" s="14" t="n"/>
+      <c r="E72" s="14" t="n"/>
+      <c r="F72" s="14" t="n"/>
+      <c r="G72" s="14" t="n"/>
+      <c r="H72" s="14" t="n"/>
+      <c r="I72" s="14" t="n"/>
+      <c r="J72" s="14" t="n"/>
+      <c r="K72" s="15" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -63898,16 +64936,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B73" s="14" t="n"/>
+      <c r="C73" s="15" t="n"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F73" s="14" t="n"/>
+      <c r="G73" s="15" t="n"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J73" s="14" t="n"/>
+      <c r="K73" s="15" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
@@ -64828,7 +65872,6 @@
         <v>-0.618</v>
       </c>
     </row>
-    <row r="133"/>
     <row r="134">
       <c r="A134" s="7" t="inlineStr">
         <is>
@@ -64979,14 +66022,22 @@
         <v>40.3414</v>
       </c>
     </row>
-    <row r="143"/>
-    <row r="144"/>
     <row r="145">
       <c r="A145" s="8" t="inlineStr">
         <is>
           <t>LOOCV (Leave-One-Out — all 84 OOF predictions in Test column)</t>
         </is>
       </c>
+      <c r="B145" s="14" t="n"/>
+      <c r="C145" s="14" t="n"/>
+      <c r="D145" s="14" t="n"/>
+      <c r="E145" s="14" t="n"/>
+      <c r="F145" s="14" t="n"/>
+      <c r="G145" s="14" t="n"/>
+      <c r="H145" s="14" t="n"/>
+      <c r="I145" s="14" t="n"/>
+      <c r="J145" s="14" t="n"/>
+      <c r="K145" s="15" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -64994,16 +66045,22 @@
           <t>Train</t>
         </is>
       </c>
+      <c r="B146" s="14" t="n"/>
+      <c r="C146" s="15" t="n"/>
       <c r="E146" s="2" t="inlineStr">
         <is>
           <t>Val</t>
         </is>
       </c>
+      <c r="F146" s="14" t="n"/>
+      <c r="G146" s="15" t="n"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
           <t>Test</t>
         </is>
       </c>
+      <c r="J146" s="14" t="n"/>
+      <c r="K146" s="15" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
@@ -66723,7 +67780,6 @@
         <v>-74.387</v>
       </c>
     </row>
-    <row r="232"/>
     <row r="233">
       <c r="A233" s="7" t="inlineStr">
         <is>

</xml_diff>